<commit_message>
feat(validation): upgrade to Auto Validate across queue, results, PDFs, and future imports (v1.1.3)
- ResultsDashboard: upgraded button to 'Auto Validate' with ShieldCheck icon
  - Full modal explaining 3-layer validation: Queue (all status), Results & PDFs, Future imports
- queue.db: validate_and_fix_queue_jobs scans and updates all jobs in SQLite in-place
- queueing: auto_fix_record_postal hook directly on enqueue_records() for all future CSV/XLSX imports
- PDF fixing: unified single-run replacement for City, State ZIP line (seamless text selection)
- open-path IPC: robust absolute path resolution against storageRootDir
</commit_message>
<xml_diff>
--- a/outputs/drive_cleaned_v2/25-09-2026_-_125_DONE/25-09-2026 - 125 DONE_CLEANED.xlsx
+++ b/outputs/drive_cleaned_v2/25-09-2026_-_125_DONE/25-09-2026 - 125 DONE_CLEANED.xlsx
@@ -526,7 +526,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>78758</t>
+          <t>78759</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -608,7 +608,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>77056</t>
+          <t>77070</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -772,7 +772,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>78212</t>
+          <t>78209</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -854,7 +854,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>77056</t>
+          <t>77090</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -936,7 +936,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>77056</t>
+          <t>77022</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1100,7 +1100,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>77056</t>
+          <t>77048</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1182,7 +1182,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>78212</t>
+          <t>78244</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1264,7 +1264,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>75208</t>
+          <t>75248</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1346,7 +1346,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>78401</t>
+          <t>78413</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1428,7 +1428,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>76111</t>
+          <t>76116</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1592,7 +1592,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>77469</t>
+          <t>77406</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1674,7 +1674,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>75040</t>
+          <t>75043</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1920,7 +1920,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>77056</t>
+          <t>77080</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2248,7 +2248,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>78758</t>
+          <t>78705</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2494,7 +2494,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>75080</t>
+          <t>75081</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -2576,7 +2576,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>77056</t>
+          <t>77084</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -2658,7 +2658,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>77494</t>
+          <t>77449</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -2740,7 +2740,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>78212</t>
+          <t>78217</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2904,7 +2904,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>92856</t>
+          <t>92867</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -3068,7 +3068,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>61614</t>
+          <t>61604</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -3232,7 +3232,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>93301</t>
+          <t>93313</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -3642,7 +3642,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>66101</t>
+          <t>66111</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -3724,7 +3724,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>63005</t>
+          <t>63011</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -4052,7 +4052,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>27403</t>
+          <t>27407</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -4134,7 +4134,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>75208</t>
+          <t>75204</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -4380,7 +4380,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>77396</t>
+          <t>77346</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -4790,7 +4790,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>60645</t>
+          <t>60644</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -4872,7 +4872,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>60645</t>
+          <t>60617</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>43085</t>
+          <t>43213</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -5036,7 +5036,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>52401</t>
+          <t>52403</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -5200,7 +5200,7 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>90024</t>
+          <t>90022</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -5282,7 +5282,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>76111</t>
+          <t>76115</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -5364,7 +5364,7 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>47713</t>
+          <t>47710</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -5610,7 +5610,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>37040</t>
+          <t>37042</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -5692,7 +5692,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>75208</t>
+          <t>75203</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -6102,7 +6102,7 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>29464</t>
+          <t>29466</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -6348,7 +6348,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>44104</t>
+          <t>44109</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -6512,7 +6512,7 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>33314</t>
+          <t>33328</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -6594,7 +6594,7 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>46226</t>
+          <t>46237</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -6758,7 +6758,7 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>92845</t>
+          <t>92840</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -6840,7 +6840,7 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>46226</t>
+          <t>46237</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -7086,7 +7086,7 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>92026</t>
+          <t>92025</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -7250,7 +7250,7 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>32835</t>
+          <t>32817</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
@@ -7332,7 +7332,7 @@
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>43085</t>
+          <t>43228</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
@@ -7496,7 +7496,7 @@
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>28269</t>
+          <t>28215</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
@@ -7824,7 +7824,7 @@
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>46226</t>
+          <t>46203</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
@@ -7906,7 +7906,7 @@
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>73034</t>
+          <t>73013</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
@@ -8316,7 +8316,7 @@
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>77377</t>
+          <t>77375</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
@@ -8398,7 +8398,7 @@
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>75208</t>
+          <t>75209</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
@@ -8644,7 +8644,7 @@
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>31901</t>
+          <t>31907</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
@@ -8890,7 +8890,7 @@
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>90024</t>
+          <t>90062</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
@@ -9054,7 +9054,7 @@
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>46038</t>
+          <t>46037</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
@@ -9300,7 +9300,7 @@
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>71129</t>
+          <t>71115</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
@@ -9464,7 +9464,7 @@
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>46226</t>
+          <t>46205</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
@@ -9710,7 +9710,7 @@
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>53401</t>
+          <t>53405</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
@@ -9792,7 +9792,7 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>73034</t>
+          <t>73013</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
@@ -10038,7 +10038,7 @@
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>67207</t>
+          <t>67205</t>
         </is>
       </c>
       <c r="G118" t="inlineStr">
@@ -10120,7 +10120,7 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>47304</t>
+          <t>47302</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
@@ -10202,7 +10202,7 @@
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>75208</t>
+          <t>75287</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
@@ -10366,7 +10366,7 @@
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>90024</t>
+          <t>90036</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
@@ -10694,7 +10694,7 @@
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>91776</t>
+          <t>91775</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">

</xml_diff>